<commit_message>
Add chart and axis titles to Excel charts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dgxa3bmKANJ93vhN2WPa2i
</commit_message>
<xml_diff>
--- a/Tehtavasarja1.xlsx
+++ b/Tehtavasarja1.xlsx
@@ -54,7 +54,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,6 +78,20 @@
       <family val="0"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -208,7 +222,41 @@
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>r(p) = -3p² + 6p - 2</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:scatterChart>
         <c:scatterStyle val="line"/>
@@ -401,13 +449,15 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="10275087"/>
-        <c:axId val="83355580"/>
+        <c:axId val="64589754"/>
+        <c:axId val="56003980"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="10275087"/>
+        <c:axId val="64589754"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="2"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -421,6 +471,121 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>hinta p</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="56003980"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="56003980"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>voitto r(p)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -447,54 +612,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83355580"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="83355580"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="10275087"/>
+        <c:crossAx val="64589754"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -527,7 +645,41 @@
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>LEGO 7674 inflaatiokorjattu hinta 2008-2025</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:scatterChart>
         <c:scatterStyle val="line"/>
@@ -702,13 +854,15 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="42602843"/>
-        <c:axId val="72958099"/>
+        <c:axId val="50220021"/>
+        <c:axId val="4218503"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="42602843"/>
+        <c:axId val="50220021"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="2025"/>
+          <c:min val="2008"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -722,6 +876,40 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>vuosi</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -748,12 +936,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72958099"/>
+        <c:crossAx val="4218503"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="72958099"/>
+        <c:axId val="4218503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -769,6 +957,40 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>hinta ($)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -795,7 +1017,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42602843"/>
+        <c:crossAx val="50220021"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>

</xml_diff>